<commit_message>
AASP01 Grupos-Usuarios: correções de consistência e novos artefatos (GQA, índice, CAP)
Traz para a gallant a versão revisada do projeto AASP01, preservando o restante
do conteúdo da branch:

- Nomes conforme MAPA-ORG-001 (Cézar Velázquez, Abraão Oliveira, Renan Kioshi,
  Caroline Jenifer).
- Siglas de processo conforme CONV-ORG-001 (REQ, VV, ITP, GPR/GCO).
- Acentuação pt-BR completa, preservando código, endpoints, nomes de
  tabela/coluna e valores de enum.
- Remoção de placeholders do corpo; meta de cobertura unificada (80%).
- Registro de Adaptação com classificação de nível (Nível 2 — Padrão).
- Novos artefatos: GQA-AASP01-001 (auditoria intermediária; auditor
  independente Silvio Baroni), 00_INDICE-AASP01 (mapa de registros) e
  CAP-AASP01-001 (capacitação da equipe).
- 21 .docx regenerados; arquivo de lock do LibreOffice removido e padrão
  adicionado ao .gitignore. Datas preservadas (projeto em aberto).

https://claude.ai/code/session_01W7xi1Lg7namhZ84Y69RKdK
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Gerenciador/AASP01_Grupos-Usuarios/GEST-AASP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Gerenciador/AASP01_Grupos-Usuarios/GEST-AASP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Abraão — Timeware Brasil</t>
+          <t>Abraão Oliveira — Timeware Brasil</t>
         </is>
       </c>
       <c r="C14" s="23" t="n"/>
@@ -823,7 +823,7 @@
       </c>
       <c r="B16" s="27" t="inlineStr">
         <is>
-          <t>Renan Kiyoshi, Henry Komatsu, Mateus Veloso — Timeware (Arquiteto/Tech Lead: Cezar Hiraki)</t>
+          <t>Renan Kioshi, Henry Komatsu, Mateus Veloso — Timeware (Arquiteto/Tech Lead: Cézar Velázquez)</t>
         </is>
       </c>
       <c r="C16" s="23" t="n"/>
@@ -2929,7 +2929,7 @@
     <row r="6" ht="27.75" customHeight="1" s="19">
       <c r="A6" s="29" t="inlineStr">
         <is>
-          <t>Abraão — Gerente de Projeto</t>
+          <t>Abraão Oliveira — Gerente de Projeto</t>
         </is>
       </c>
       <c r="B6" s="29" t="inlineStr">
@@ -2966,7 +2966,7 @@
     <row r="7" ht="27.75" customHeight="1" s="19">
       <c r="A7" s="29" t="inlineStr">
         <is>
-          <t>Cezar Hiraki — Arquiteto / Tech Lead / DevOps / Revisor de PRs</t>
+          <t>Cézar Velázquez — Arquiteto / Tech Lead / DevOps / Revisor de PRs</t>
         </is>
       </c>
       <c r="B7" s="29" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>Devs: Renan Kiyoshi, Henry Komatsu, Mateus Veloso · QA: Caroline Sousa · GQA: Jonathan</t>
+          <t>Devs: Renan Kioshi, Henry Komatsu, Mateus Veloso · QA: Caroline Jenifer · GQA: Silvio Baroni (auditor independente — Time de Melhoria Contínua)</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="B10" s="30" t="inlineStr">
         <is>
-          <t>Sobrecarga ou indisponibilidade de Cezar Hiraki, que acumula papéis técnicos (Arquiteto/Tech Lead/DevOps/Revisor/GCO)</t>
+          <t>Sobrecarga ou indisponibilidade de Cézar Velázquez, que acumula papéis técnicos (Arquiteto/Tech Lead/DevOps/Revisor/GCO)</t>
         </is>
       </c>
       <c r="C10" s="30" t="n">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="G10" s="30" t="inlineStr">
         <is>
-          <t>Documentação técnica mantida atualizada; pair programming com Renan Kiyoshi para transferência de conhecimento</t>
+          <t>Documentação técnica mantida atualizada; pair programming com Renan Kioshi para transferência de conhecimento</t>
         </is>
       </c>
       <c r="H10" s="30" t="inlineStr">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="J10" s="30" t="inlineStr">
         <is>
-          <t>Contingência: equipe de 3 devs (Renan, Henry, Mateus Veloso) absorve a carga; Renan Kiyoshi preparado para assumir GCO</t>
+          <t>Contingência: equipe de 3 devs (Renan, Henry, Mateus Veloso) absorve a carga; Renan Kioshi preparado para assumir GCO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(AASP01): alinha a API real (GerenciarGruposController, HTTP 200/400, funcao), Azure->GitLab (MR !1-!7) e ortografia PT-BR
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Gerenciador/AASP01_Grupos-Usuarios/GEST-AASP01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Gerenciador/AASP01_Grupos-Usuarios/GEST-AASP01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -623,7 +623,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -764,7 +763,6 @@
       <c r="G11" s="23" t="n"/>
       <c r="H11" s="23" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="19">
       <c r="A13" s="22" t="inlineStr">
         <is>
@@ -833,7 +831,6 @@
       <c r="G16" s="23" t="n"/>
       <c r="H16" s="23" t="n"/>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="19">
       <c r="A18" s="22" t="inlineStr">
         <is>
@@ -902,7 +899,6 @@
       <c r="G21" s="23" t="n"/>
       <c r="H21" s="23" t="n"/>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="19">
       <c r="A23" s="22" t="inlineStr">
         <is>
@@ -1088,11 +1084,10 @@
     <row r="2" ht="15" customHeight="1" s="19">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>Fonte: CTQ-AASP01-001 · REL-VV-AASP01-001 · VV-AASP01-001  |  10 cenários Sprint 1 (✅); Sprint 2–4 a executar</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Fonte: CTQ-AASP01-001 · REL-VV-AASP01-001 · VV-AASP01-001  |  10 cenários Sprint 1 (✅); Sprint 2–3 a executar</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -1179,18 +1174,17 @@
       </c>
       <c r="E6" s="36" t="inlineStr">
         <is>
-          <t>usuário autenticado com permissão de administrador</t>
+          <t>usuário autenticado; nenhum grupo 'Gestores' no escritório</t>
         </is>
       </c>
       <c r="F6" s="36" t="inlineStr">
         <is>
-          <t>envia POST /grupos com nome e descrição válidos</t>
+          <t>envia POST incluirgrupo com {nome:'Gestores', grupoDeUsuarios:[]}</t>
         </is>
       </c>
       <c r="G6" s="36" t="inlineStr">
         <is>
-          <t>grupo criado com id gerado
-E status 201 retornado</t>
+          <t>status 200; Sucesso=true; MensagemPublica='Grupo incluido com sucesso'</t>
         </is>
       </c>
       <c r="H6" s="36" t="inlineStr">
@@ -1198,11 +1192,7 @@
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I6" s="36" t="inlineStr">
-        <is>
-          <t>Coberto por 3 testes unitários</t>
-        </is>
-      </c>
+      <c r="I6" s="36" t="inlineStr"/>
     </row>
     <row r="7" ht="39.75" customHeight="1" s="19">
       <c r="A7" s="36" t="inlineStr">
@@ -1218,7 +1208,7 @@
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
-          <t>Listar todos os grupos ativos — happy path</t>
+          <t>Listar grupos — happy path</t>
         </is>
       </c>
       <c r="D7" s="36" t="inlineStr">
@@ -1228,18 +1218,17 @@
       </c>
       <c r="E7" s="36" t="inlineStr">
         <is>
-          <t>existem grupos cadastrados no banco auxo3</t>
+          <t>existem grupos com excluido=0 no escritório</t>
         </is>
       </c>
       <c r="F7" s="36" t="inlineStr">
         <is>
-          <t>envia GET /grupos</t>
+          <t>envia GET listargrupo (paginado)</t>
         </is>
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t>retorna lista de grupos com id, nome, status
-E status 200</t>
+          <t>status 200; RetornaDados com a lista de grupos</t>
         </is>
       </c>
       <c r="H7" s="36" t="inlineStr">
@@ -1247,7 +1236,7 @@
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I7" s="36" t="n"/>
+      <c r="I7" s="36" t="inlineStr"/>
     </row>
     <row r="8" ht="39.75" customHeight="1" s="19">
       <c r="A8" s="36" t="inlineStr">
@@ -1263,7 +1252,7 @@
       </c>
       <c r="C8" s="36" t="inlineStr">
         <is>
-          <t>Atualizar nome do grupo — happy path</t>
+          <t>Consultar usuários de um grupo — happy path</t>
         </is>
       </c>
       <c r="D8" s="36" t="inlineStr">
@@ -1273,18 +1262,17 @@
       </c>
       <c r="E8" s="36" t="inlineStr">
         <is>
-          <t>grupo com id 5 existe e está ativo</t>
+          <t>grupo id 5 possui membros</t>
         </is>
       </c>
       <c r="F8" s="36" t="inlineStr">
         <is>
-          <t>envia PUT /grupos/5 com novo nome</t>
+          <t>envia GET buscargrupoporid (id 5)</t>
         </is>
       </c>
       <c r="G8" s="36" t="inlineStr">
         <is>
-          <t>grupo atualizado
-E status 200 retornado</t>
+          <t>status 200; RetornaDados com os usuários e funções do grupo</t>
         </is>
       </c>
       <c r="H8" s="36" t="inlineStr">
@@ -1292,7 +1280,7 @@
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I8" s="36" t="n"/>
+      <c r="I8" s="36" t="inlineStr"/>
     </row>
     <row r="9" ht="39.75" customHeight="1" s="19">
       <c r="A9" s="36" t="inlineStr">
@@ -1308,7 +1296,7 @@
       </c>
       <c r="C9" s="36" t="inlineStr">
         <is>
-          <t>Exclusão lógica (soft delete) de grupo — happy path</t>
+          <t>Alterar grupo — happy path</t>
         </is>
       </c>
       <c r="D9" s="36" t="inlineStr">
@@ -1318,19 +1306,17 @@
       </c>
       <c r="E9" s="36" t="inlineStr">
         <is>
-          <t>grupo com id 7 existe e não possui usuários vinculados</t>
+          <t>grupo id 5 existe</t>
         </is>
       </c>
       <c r="F9" s="36" t="inlineStr">
         <is>
-          <t>envia DELETE /grupos/7</t>
+          <t>envia POST alterargrupo com {id:5, nome:'Gestores Senior', grupoDeUsuarios:[...]}</t>
         </is>
       </c>
       <c r="G9" s="36" t="inlineStr">
         <is>
-          <t>campo ativo = false no banco
-E status 204 retornado
-E grupo não aparece em GET /grupos</t>
+          <t>status 200; data_alteracao atualizada</t>
         </is>
       </c>
       <c r="H9" s="36" t="inlineStr">
@@ -1338,11 +1324,7 @@
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I9" s="36" t="inlineStr">
-        <is>
-          <t>Soft delete validado no banco</t>
-        </is>
-      </c>
+      <c r="I9" s="36" t="inlineStr"/>
     </row>
     <row r="10" ht="39.75" customHeight="1" s="19">
       <c r="A10" s="36" t="inlineStr">
@@ -1358,28 +1340,27 @@
       </c>
       <c r="C10" s="36" t="inlineStr">
         <is>
-          <t>Tentar criar grupo com nome duplicado — sad path</t>
+          <t>Excluir grupo (soft delete) — happy path</t>
         </is>
       </c>
       <c r="D10" s="36" t="inlineStr">
         <is>
-          <t>Sad</t>
+          <t>Happy</t>
         </is>
       </c>
       <c r="E10" s="36" t="inlineStr">
         <is>
-          <t>grupo com nome 'Administradores' já existe</t>
+          <t>grupo id 7 existe</t>
         </is>
       </c>
       <c r="F10" s="36" t="inlineStr">
         <is>
-          <t>envia POST /grupos com nome 'Administradores'</t>
+          <t>envia POST excluirgrupo com {id:7, notificarMembros:false}</t>
         </is>
       </c>
       <c r="G10" s="36" t="inlineStr">
         <is>
-          <t>status 409 retornado
-E mensagem 'Nome de grupo já existe'</t>
+          <t>status 200; excluido=1 no banco; não aparece em listargrupo</t>
         </is>
       </c>
       <c r="H10" s="36" t="inlineStr">
@@ -1389,25 +1370,25 @@
       </c>
       <c r="I10" s="36" t="inlineStr">
         <is>
-          <t>Validação de unicidade</t>
+          <t>Soft delete validado no banco</t>
         </is>
       </c>
     </row>
     <row r="11" ht="39.75" customHeight="1" s="19">
       <c r="A11" s="36" t="inlineStr">
         <is>
-          <t>AG-21
-Permissões</t>
+          <t>AG-20
+CRUD Grupos</t>
         </is>
       </c>
       <c r="B11" s="36" t="inlineStr">
         <is>
-          <t>PERM-01</t>
+          <t>GRP-06</t>
         </is>
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Associar permissões válidas a grupo — happy path</t>
+          <t>Ativar/desativar grupo — happy path</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -1417,19 +1398,17 @@
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
-          <t>grupo id 3 existe
-E permissões ['leitura','escrita'] são válidas</t>
+          <t>grupo id 5 existe</t>
         </is>
       </c>
       <c r="F11" s="36" t="inlineStr">
         <is>
-          <t>envia PUT /grupos/3/permissoes com lista de permissões</t>
+          <t>envia POST ativardesativar com {id:5, ativo:0}</t>
         </is>
       </c>
       <c r="G11" s="36" t="inlineStr">
         <is>
-          <t>permissões associadas ao grupo
-E status 200 retornado</t>
+          <t>status 200; campo ativo atualizado para 0</t>
         </is>
       </c>
       <c r="H11" s="36" t="inlineStr">
@@ -1437,23 +1416,23 @@
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I11" s="36" t="n"/>
+      <c r="I11" s="36" t="inlineStr"/>
     </row>
     <row r="12" ht="39.75" customHeight="1" s="19">
       <c r="A12" s="36" t="inlineStr">
         <is>
-          <t>AG-21
-Permissões</t>
+          <t>AG-20
+CRUD Grupos</t>
         </is>
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>PERM-02</t>
+          <t>GRP-07</t>
         </is>
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Tentar associar permissão inexistente — sad path</t>
+          <t>Criar grupo com nome duplicado — sad path</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -1463,18 +1442,17 @@
       </c>
       <c r="E12" s="36" t="inlineStr">
         <is>
-          <t>grupo id 3 existe</t>
+          <t>grupo 'Administradores' já existe no escritório</t>
         </is>
       </c>
       <c r="F12" s="36" t="inlineStr">
         <is>
-          <t>envia PUT /grupos/3/permissoes com permissão 'superadmin' inválida</t>
+          <t>envia POST incluirgrupo com {nome:'Administradores'}</t>
         </is>
       </c>
       <c r="G12" s="36" t="inlineStr">
         <is>
-          <t>status 400 retornado
-E mensagem de validação de permissão inválida</t>
+          <t>status 400; Sucesso=false; MensagemPublica='Grupo ja existe'</t>
         </is>
       </c>
       <c r="H12" s="36" t="inlineStr">
@@ -1482,159 +1460,144 @@
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I12" s="36" t="inlineStr">
-        <is>
-          <t>Validação de enum</t>
-        </is>
-      </c>
+      <c r="I12" s="36" t="inlineStr"/>
     </row>
     <row r="13" ht="39.75" customHeight="1" s="19">
       <c r="A13" s="36" t="inlineStr">
         <is>
+          <t>AG-21
+Função</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>FUNC-01</t>
+        </is>
+      </c>
+      <c r="C13" s="36" t="inlineStr">
+        <is>
+          <t>Alterar função do usuário no grupo — happy path</t>
+        </is>
+      </c>
+      <c r="D13" s="36" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E13" s="36" t="inlineStr">
+        <is>
+          <t>usuário 42 é membro do grupo (função Usuario)</t>
+        </is>
+      </c>
+      <c r="F13" s="36" t="inlineStr">
+        <is>
+          <t>envia POST alterarfuncaodousuario com {usuarioId:42, funcaoId:1, funcao:1}</t>
+        </is>
+      </c>
+      <c r="G13" s="36" t="inlineStr">
+        <is>
+          <t>status 200; função atualizada para Administrador</t>
+        </is>
+      </c>
+      <c r="H13" s="36" t="inlineStr">
+        <is>
+          <t>✅ OK</t>
+        </is>
+      </c>
+      <c r="I13" s="36" t="inlineStr"/>
+    </row>
+    <row r="14" ht="39.75" customHeight="1" s="19">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
           <t>AG-22
 Vínculos</t>
         </is>
       </c>
-      <c r="B13" s="36" t="inlineStr">
+      <c r="B14" s="36" t="inlineStr">
         <is>
           <t>VINC-01</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
-        <is>
-          <t>Vincular usuário a grupo — happy path</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
+      <c r="C14" s="36" t="inlineStr">
+        <is>
+          <t>Vincular usuários ao grupo — happy path</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
         <is>
           <t>Happy</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>usuário id 42 existe
-E grupo id 3 existe e está ativo</t>
-        </is>
-      </c>
-      <c r="F13" s="36" t="inlineStr">
-        <is>
-          <t>envia POST /grupos/3/usuarios com { 'usuarioId': 42 }</t>
-        </is>
-      </c>
-      <c r="G13" s="36" t="inlineStr">
-        <is>
-          <t>vínculo criado
-E status 201 retornado</t>
-        </is>
-      </c>
-      <c r="H13" s="36" t="inlineStr">
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>grupo id 3 existe; usuários 42 e 711 existem</t>
+        </is>
+      </c>
+      <c r="F14" s="36" t="inlineStr">
+        <is>
+          <t>envia POST alterargrupo com grupoDeUsuarios:[{id:42,funcaoId:0},{id:711,funcaoId:1}]</t>
+        </is>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>status 200; vínculos criados em grupos_usuarios_vinculos</t>
+        </is>
+      </c>
+      <c r="H14" s="36" t="inlineStr">
         <is>
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I13" s="36" t="n"/>
-    </row>
-    <row r="14" ht="39.75" customHeight="1" s="19">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="I14" s="36" t="inlineStr"/>
+    </row>
+    <row r="15" ht="39.75" customHeight="1" s="19">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>AG-22
 Vínculos</t>
         </is>
       </c>
-      <c r="B14" s="36" t="inlineStr">
+      <c r="B15" s="36" t="inlineStr">
         <is>
           <t>VINC-02</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
-        <is>
-          <t>Desvincular usuário de grupo — happy path</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
+      <c r="C15" s="36" t="inlineStr">
+        <is>
+          <t>Remover usuário do grupo — happy path</t>
+        </is>
+      </c>
+      <c r="D15" s="36" t="inlineStr">
         <is>
           <t>Happy</t>
         </is>
       </c>
-      <c r="E14" s="36" t="inlineStr">
-        <is>
-          <t>usuário id 42 está vinculado ao grupo id 3</t>
-        </is>
-      </c>
-      <c r="F14" s="36" t="inlineStr">
-        <is>
-          <t>envia DELETE /grupos/3/usuarios/42</t>
-        </is>
-      </c>
-      <c r="G14" s="36" t="inlineStr">
-        <is>
-          <t>vínculo removido
-E status 204 retornado
-E usuário não aparece em GET /grupos/3/usuarios</t>
-        </is>
-      </c>
-      <c r="H14" s="36" t="inlineStr">
+      <c r="E15" s="36" t="inlineStr">
+        <is>
+          <t>usuário 711 vinculado ao grupo 3</t>
+        </is>
+      </c>
+      <c r="F15" s="36" t="inlineStr">
+        <is>
+          <t>envia POST removerusuario com {id:711, grupoId:3}</t>
+        </is>
+      </c>
+      <c r="G15" s="36" t="inlineStr">
+        <is>
+          <t>status 200; excluido=1 no vínculo; some de buscargrupoporid</t>
+        </is>
+      </c>
+      <c r="H15" s="36" t="inlineStr">
         <is>
           <t>✅ OK</t>
         </is>
       </c>
-      <c r="I14" s="36" t="n"/>
-    </row>
-    <row r="15" ht="39.75" customHeight="1" s="19">
-      <c r="A15" s="36" t="inlineStr">
-        <is>
-          <t>AG-22
-Vínculos</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="inlineStr">
-        <is>
-          <t>VINC-03</t>
-        </is>
-      </c>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>Tentar vincular usuário inexistente — sad path</t>
-        </is>
-      </c>
-      <c r="D15" s="36" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="E15" s="36" t="inlineStr">
-        <is>
-          <t>grupo id 3 existe
-E usuário id 999 não existe no banco</t>
-        </is>
-      </c>
-      <c r="F15" s="36" t="inlineStr">
-        <is>
-          <t>envia POST /grupos/3/usuarios com { 'usuarioId': 999 }</t>
-        </is>
-      </c>
-      <c r="G15" s="36" t="inlineStr">
-        <is>
-          <t>status 404 retornado
-E mensagem 'Usuário não encontrado'</t>
-        </is>
-      </c>
-      <c r="H15" s="36" t="inlineStr">
-        <is>
-          <t>✅ OK</t>
-        </is>
-      </c>
-      <c r="I15" s="36" t="inlineStr">
-        <is>
-          <t>FK validada no Dapper</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
+      <c r="I15" s="36" t="inlineStr"/>
+    </row>
     <row r="17" ht="15" customHeight="1" s="19">
       <c r="A17" s="22" t="inlineStr">
         <is>
-          <t>CENÁRIOS DE TESTE — SPRINT 2+ (AG-23, AG-24, AG-25) — A EXECUTAR</t>
+          <t>CENÁRIOS DE TESTE — SPRINT 2-3 (AG-23, AG-24, AG-25) — PLANEJADO / A EXECUTAR</t>
         </is>
       </c>
       <c r="B17" s="23" t="n"/>
@@ -1717,17 +1680,17 @@
       </c>
       <c r="E19" s="37" t="inlineStr">
         <is>
-          <t>grupo criado com sucesso via POST /grupos</t>
+          <t>(planejado — Sprint 2) ao criar/alterar um grupo</t>
         </is>
       </c>
       <c r="F19" s="37" t="inlineStr">
         <is>
-          <t>operação é concluída</t>
+          <t>(planejado) operação de escrita em grupo</t>
         </is>
       </c>
       <c r="G19" s="37" t="inlineStr">
         <is>
-          <t>registro inserido em AuditoriaGrupos com usuário, timestamp e ação='CREATE'</t>
+          <t>(planejado) registro de auditoria com usuário, timestamp e ação</t>
         </is>
       </c>
       <c r="H19" s="37" t="inlineStr">
@@ -1796,7 +1759,7 @@
       </c>
       <c r="C21" s="37" t="inlineStr">
         <is>
-          <t>Listar grupos com usuários e permissões — happy path</t>
+          <t>Relatório consolidado de grupos e membros — happy path</t>
         </is>
       </c>
       <c r="D21" s="37" t="inlineStr">
@@ -1806,18 +1769,17 @@
       </c>
       <c r="E21" s="37" t="inlineStr">
         <is>
-          <t>existem grupos com usuários e permissões cadastrados</t>
+          <t>(planejado — Sprint 3) existem grupos com membros cadastrados</t>
         </is>
       </c>
       <c r="F21" s="37" t="inlineStr">
         <is>
-          <t>envia GET /grupos/relatorio</t>
+          <t>(planejado) consulta o relatório consolidado</t>
         </is>
       </c>
       <c r="G21" s="37" t="inlineStr">
         <is>
-          <t>retorna lista consolidada com grupos, membros e permissões
-E status 200</t>
+          <t>(planejado) retorna relatório consolidado de grupos e membros</t>
         </is>
       </c>
       <c r="H21" s="37" t="inlineStr">
@@ -1872,7 +1834,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -1971,7 +1932,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="19">
       <c r="A8" s="22" t="inlineStr">
         <is>
@@ -2054,7 +2014,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>AG-20 (CRUD Grupos), AG-21 (Permissões), AG-22 (Vínculo Usuário↔Grupo); endpoints POST/GET/PUT/DELETE; testes unitários</t>
+          <t>AG-20 (CRUD Grupos), AG-21 (Função), AG-22 (Vínculo Usuário↔Grupo); endpoints GET/POST (api/gerenciar/grupos); testes unitários</t>
         </is>
       </c>
       <c r="G10" s="30" t="inlineStr">
@@ -2145,34 +2105,12 @@
       <c r="H12" s="29" t="n"/>
     </row>
     <row r="13" ht="27.75" customHeight="1" s="19">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Sprint 4 (Encerramento)</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>07/07/2026</t>
-        </is>
-      </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>11/07/2026</t>
-        </is>
-      </c>
-      <c r="D13" s="29" t="inlineStr">
-        <is>
-          <t>1 semana</t>
-        </is>
-      </c>
-      <c r="E13" s="29" t="n">
-        <v>8</v>
-      </c>
-      <c r="F13" s="29" t="inlineStr">
-        <is>
-          <t>Homologação final; TAE; LI; GQA; entrega formal</t>
-        </is>
-      </c>
+      <c r="A13" s="29" t="n"/>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="29" t="n"/>
       <c r="G13" s="29" t="inlineStr">
         <is>
           <t>📅 Planejado</t>
@@ -2184,7 +2122,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="19">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -2303,7 +2240,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -2374,7 +2310,7 @@
       </c>
       <c r="B6" s="30" t="inlineStr">
         <is>
-          <t>CRUD de Grupos de Usuários — criação, leitura, atualização e exclusão lógica (soft delete) de grupos; endpoints RESTful POST /grupos, GET /grupos, GET /grupos/{id}, PUT /grupos/{id}, DELETE /grupos/{id}</t>
+          <t>CRUD de Grupos de Usuários — criação, listagem, consulta, alteração, exclusão lógica (soft delete) e ativação/desativação; endpoints incluirgrupo, listargrupo, buscargrupoporid, alterargrupo, excluirgrupo, ativardesativar (api/gerenciar/grupos)</t>
         </is>
       </c>
       <c r="C6" s="30" t="inlineStr">
@@ -2419,7 +2355,7 @@
       </c>
       <c r="B7" s="30" t="inlineStr">
         <is>
-          <t>Permissões por Grupo — associação de permissões a grupos; controle de acesso baseado em grupo (RBAC); endpoint PUT /grupos/{id}/permissoes</t>
+          <t>Função do Usuário no Grupo — definição do papel do usuário (Usuario/Administrador); endpoint alterarfuncaodousuario</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
@@ -2464,7 +2400,7 @@
       </c>
       <c r="B8" s="30" t="inlineStr">
         <is>
-          <t>Vinculação Usuário ↔ Grupo — adição e remoção de usuários em grupos; endpoint POST /grupos/{id}/usuarios e DELETE /grupos/{id}/usuarios/{userId}</t>
+          <t>Vinculação Usuário ↔ Grupo — usuários enviados na lista grupoDeUsuarios de incluirgrupo/alterargrupo; remoção via removerusuario</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
@@ -2509,7 +2445,7 @@
       </c>
       <c r="B9" s="31" t="inlineStr">
         <is>
-          <t>Auditoria e Log de Ações — registro de todas as operações em grupos/permissões com usuário, timestamp e ação; tabela AuditoriaGrupos no banco auxo3</t>
+          <t>Auditoria e Log de Ações (planejado — Sprint 2) — registro das operações de escrita em grupos com usuário, timestamp e ação</t>
         </is>
       </c>
       <c r="C9" s="31" t="inlineStr">
@@ -2554,7 +2490,7 @@
       </c>
       <c r="B10" s="31" t="inlineStr">
         <is>
-          <t>Integração ms.temis.vinculos — sincronização bidirecional de vínculos entre Grupos (auxo3) e Vínculos (temis3); chamadas HTTP entre microsserviços</t>
+          <t>Integração ms.temis.vinculos (planejado — Sprint 2) — sincronização de vínculos entre auxo3 e temis3 via HTTP</t>
         </is>
       </c>
       <c r="C10" s="31" t="inlineStr">
@@ -2599,7 +2535,7 @@
       </c>
       <c r="B11" s="29" t="inlineStr">
         <is>
-          <t>Relatórios de Grupos — endpoints de consulta consolidada; listagem de grupos com usuários e permissões; filtros por status e tipo; exportação CSV</t>
+          <t>Relatórios de Grupos (planejado — Sprint 3) — consulta consolidada de grupos e membros; exportação CSV</t>
         </is>
       </c>
       <c r="C11" s="29" t="inlineStr">
@@ -2632,7 +2568,6 @@
       </c>
       <c r="I11" s="29" t="n"/>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="19">
       <c r="A13" s="22" t="inlineStr">
         <is>
@@ -2875,7 +2810,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -3208,7 +3142,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -3415,22 +3348,10 @@
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1" s="19">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>07/07–11/07/2026</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="29" t="n">
-        <v>8</v>
-      </c>
+      <c r="A9" s="29" t="n"/>
+      <c r="B9" s="29" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
       <c r="E9" s="29" t="inlineStr">
         <is>
           <t>—</t>
@@ -3462,7 +3383,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="19">
       <c r="A11" s="22" t="inlineStr">
         <is>
@@ -3587,7 +3507,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -3939,7 +3858,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -4055,7 +3973,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="22" t="inlineStr">
         <is>
@@ -4446,7 +4363,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="19">
       <c r="A4" s="25" t="inlineStr">
         <is>
@@ -4509,7 +4425,7 @@
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>⏳ Auditorias agendadas para Sprint 3 e encerramento (Sprint 4)</t>
+          <t>⏳ Auditorias agendadas para a Sprint 3 (encerramento)</t>
         </is>
       </c>
       <c r="C7" s="23" t="n"/>
@@ -4519,7 +4435,6 @@
       <c r="G7" s="23" t="n"/>
       <c r="H7" s="23" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="19">
       <c r="A9" s="22" t="inlineStr">
         <is>
@@ -4631,7 +4546,7 @@
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="D12" s="31" t="inlineStr">
@@ -4660,7 +4575,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="24" customHeight="1" s="19">
       <c r="A14" s="35" t="inlineStr">
         <is>

</xml_diff>